<commit_message>
chore: snapshot current workspace changes
</commit_message>
<xml_diff>
--- a/plant-thesis/08_参考文献/参考文献核对表.xlsx
+++ b/plant-thesis/08_参考文献/参考文献核对表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\zhishi-plant-system\plant-thesis\08_参考文献\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE69486D-A73E-49B9-AB7C-5B58BBFF47F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C91B31-557C-463D-A1F4-4B7861984602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>编号</t>
   </si>
@@ -39,12 +39,21 @@
     <t>是否已引用</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>Citizen Science: A Developing Tool for Expanding Science Knowledge and Scientific Literacy | BioScience | Oxford Academic</t>
+  </si>
+  <si>
+    <t>Bonney R, et al. Citizen Science: A Developing Tool for Expanding Science Knowledge[J]. BioScience, 2021.</t>
+  </si>
+  <si>
+    <t>公民科学动员公众在长时间内收集大量数据，覆盖多种栖息地和地点。公民科学项目在推动科学知识方面取得了显著成功，公民科学家的贡献现为全球物种的出现和分布提供了大量数据。大多数公民科学项目还致力于帮助参与者了解他们观察到的生物体，并体验科学调查的过程。开发和实施能够带来科学和教育成果的公共数据收集项目需要大量努力。本文描述了康奈尔鸟类学实验室在过去二十年中发展起来的公民科学项目构建和运营模式。我们希望我们的模型能够为生物多样性监测、生物研究和科学教育领域提供参考，同时为公民科学文化提供窗口。</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,6 +75,20 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -84,21 +107,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -363,10 +396,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -381,10 +414,28 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="F4" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" location="no-access-message" display="https://academic.oup.com/bioscience/article-abstract/59/11/977/251421?login=false - no-access-message" xr:uid="{F6D1E31C-4DBD-48F6-9268-96B06C6B0C80}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -393,7 +444,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -404,7 +455,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>